<commit_message>
modified:   jsd-solar-inverter.yaml Config and settings sensors were added
</commit_message>
<xml_diff>
--- a/docs/INV-Modbus地址表3KU（外发）V1.20.xlsx
+++ b/docs/INV-Modbus地址表3KU（外发）V1.20.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Downloads\Invertor-BMS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\home\VSCode\ESPHome_JSDSolar_inverter\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4755" tabRatio="849" firstSheet="1" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" tabRatio="849" firstSheet="12" activeTab="21"/>
   </bookViews>
   <sheets>
     <sheet name=" Version information" sheetId="20" r:id="rId1"/>
@@ -2465,9 +2465,6 @@
     <t>constant pressure point</t>
   </si>
   <si>
-    <t>Lead-acid: 56.4V; Non-adjustable water-filled: 58V; Non-adjustable ternary lithium/lithium iron phosphate/custom: 48V-60V</t>
-  </si>
-  <si>
     <t>float point</t>
   </si>
   <si>
@@ -2799,6 +2796,9 @@
   </si>
   <si>
     <t>24</t>
+  </si>
+  <si>
+    <t>Non-adjustable Lead-acid: 56.4V; Non-adjustable water-filled: 58V; ternary lithium 48V-60V/lithium iron phosphate/custom: 50V-58V</t>
   </si>
 </sst>
 </file>
@@ -3387,46 +3387,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3438,13 +3408,43 @@
     <xf numFmtId="49" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4275,8 +4275,9 @@
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="5.5703125" customWidth="1"/>
     <col min="4" max="4" width="7.5703125" customWidth="1"/>
-    <col min="5" max="5" width="5.5703125" customWidth="1"/>
-    <col min="6" max="7" width="17.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="46.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" customWidth="1"/>
     <col min="8" max="8" width="5.5703125" style="3" customWidth="1"/>
     <col min="9" max="9" width="5.5703125" customWidth="1"/>
     <col min="10" max="11" width="7.5703125" customWidth="1"/>
@@ -5828,7 +5829,8 @@
     <col min="3" max="3" width="5.5703125" customWidth="1"/>
     <col min="4" max="4" width="7.5703125" customWidth="1"/>
     <col min="5" max="5" width="5.5703125" customWidth="1"/>
-    <col min="6" max="7" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="33" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
     <col min="8" max="9" width="5.5703125" customWidth="1"/>
     <col min="10" max="11" width="7.5703125" customWidth="1"/>
   </cols>
@@ -10772,7 +10774,7 @@
     <col min="3" max="3" width="23.28515625" customWidth="1"/>
     <col min="4" max="4" width="39.85546875" style="28" customWidth="1"/>
     <col min="5" max="5" width="18.140625" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" customWidth="1"/>
     <col min="7" max="7" width="18.140625" customWidth="1"/>
     <col min="8" max="8" width="15.28515625" customWidth="1"/>
     <col min="9" max="9" width="28.5703125" customWidth="1"/>
@@ -11242,7 +11244,8 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.140625" customWidth="1"/>
-    <col min="6" max="7" width="26.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.7109375" customWidth="1"/>
+    <col min="7" max="7" width="26.28515625" customWidth="1"/>
     <col min="9" max="9" width="17.42578125" customWidth="1"/>
     <col min="12" max="12" width="8.7109375" style="31"/>
     <col min="13" max="13" width="8.7109375" style="22"/>
@@ -13596,27 +13599,27 @@
       <c r="C1" s="65">
         <v>1</v>
       </c>
-      <c r="D1" s="96">
+      <c r="D1" s="114">
         <v>2</v>
       </c>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96">
+      <c r="E1" s="114"/>
+      <c r="F1" s="114">
         <v>2</v>
       </c>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96">
+      <c r="G1" s="114"/>
+      <c r="H1" s="114">
         <v>2</v>
       </c>
-      <c r="I1" s="96"/>
+      <c r="I1" s="114"/>
     </row>
     <row r="2" spans="1:22" ht="27.95" customHeight="1">
-      <c r="A2" s="115" t="s">
+      <c r="A2" s="99" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="115" t="s">
+      <c r="B2" s="99" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="115" t="s">
+      <c r="C2" s="99" t="s">
         <v>55</v>
       </c>
       <c r="D2" s="67" t="s">
@@ -13625,7 +13628,7 @@
       <c r="E2" s="67" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="115" t="s">
+      <c r="F2" s="99" t="s">
         <v>57</v>
       </c>
       <c r="G2" s="116" t="s">
@@ -13639,16 +13642,16 @@
       </c>
     </row>
     <row r="3" spans="1:22" ht="16.350000000000001" customHeight="1">
-      <c r="A3" s="115"/>
-      <c r="B3" s="115"/>
-      <c r="C3" s="115"/>
+      <c r="A3" s="99"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="99"/>
       <c r="D3" s="66" t="s">
         <v>60</v>
       </c>
       <c r="E3" s="66" t="s">
         <v>61</v>
       </c>
-      <c r="F3" s="115"/>
+      <c r="F3" s="99"/>
       <c r="G3" s="116"/>
       <c r="H3" s="66" t="s">
         <v>61</v>
@@ -13694,84 +13697,84 @@
       <c r="A9" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="97" t="s">
+      <c r="B9" s="115" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="97"/>
-      <c r="D9" s="97"/>
-      <c r="E9" s="97"/>
+      <c r="C9" s="115"/>
+      <c r="D9" s="115"/>
+      <c r="E9" s="115"/>
     </row>
     <row r="10" spans="1:22">
       <c r="A10" s="75">
         <v>1</v>
       </c>
-      <c r="B10" s="98" t="s">
+      <c r="B10" s="113" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
     </row>
     <row r="11" spans="1:22">
       <c r="A11" s="75">
         <v>2</v>
       </c>
-      <c r="B11" s="98" t="s">
+      <c r="B11" s="113" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="98"/>
-      <c r="D11" s="98"/>
-      <c r="E11" s="98"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="113"/>
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="75">
         <v>3</v>
       </c>
-      <c r="B12" s="98" t="s">
+      <c r="B12" s="113" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="98"/>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
+      <c r="C12" s="113"/>
+      <c r="D12" s="113"/>
+      <c r="E12" s="113"/>
     </row>
     <row r="13" spans="1:22">
       <c r="A13" s="76">
         <v>4</v>
       </c>
-      <c r="B13" s="98" t="s">
+      <c r="B13" s="113" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="98"/>
-      <c r="D13" s="98"/>
-      <c r="E13" s="98"/>
+      <c r="C13" s="113"/>
+      <c r="D13" s="113"/>
+      <c r="E13" s="113"/>
     </row>
     <row r="15" spans="1:22">
-      <c r="A15" s="99" t="s">
+      <c r="A15" s="107" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="99"/>
-      <c r="C15" s="99"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="99"/>
-      <c r="F15" s="99"/>
-      <c r="G15" s="99"/>
-      <c r="H15" s="99"/>
-      <c r="I15" s="99"/>
+      <c r="B15" s="107"/>
+      <c r="C15" s="107"/>
+      <c r="D15" s="107"/>
+      <c r="E15" s="107"/>
+      <c r="F15" s="107"/>
+      <c r="G15" s="107"/>
+      <c r="H15" s="107"/>
+      <c r="I15" s="107"/>
       <c r="J15" s="83"/>
-      <c r="K15" s="100" t="s">
+      <c r="K15" s="108" t="s">
         <v>75</v>
       </c>
-      <c r="L15" s="100"/>
-      <c r="M15" s="100"/>
-      <c r="N15" s="100"/>
-      <c r="O15" s="100"/>
-      <c r="P15" s="100"/>
-      <c r="Q15" s="100"/>
-      <c r="R15" s="100"/>
-      <c r="S15" s="100"/>
-      <c r="T15" s="100"/>
-      <c r="U15" s="100"/>
-      <c r="V15" s="100"/>
+      <c r="L15" s="108"/>
+      <c r="M15" s="108"/>
+      <c r="N15" s="108"/>
+      <c r="O15" s="108"/>
+      <c r="P15" s="108"/>
+      <c r="Q15" s="108"/>
+      <c r="R15" s="108"/>
+      <c r="S15" s="108"/>
+      <c r="T15" s="108"/>
+      <c r="U15" s="108"/>
+      <c r="V15" s="108"/>
     </row>
     <row r="16" spans="1:22" ht="24">
       <c r="A16" s="77" t="s">
@@ -13783,18 +13786,18 @@
       <c r="C16" s="78">
         <v>1</v>
       </c>
-      <c r="D16" s="101">
+      <c r="D16" s="110">
         <v>2</v>
       </c>
-      <c r="E16" s="101"/>
-      <c r="F16" s="101">
+      <c r="E16" s="110"/>
+      <c r="F16" s="110">
         <v>2</v>
       </c>
-      <c r="G16" s="101"/>
-      <c r="H16" s="101">
+      <c r="G16" s="110"/>
+      <c r="H16" s="110">
         <v>2</v>
       </c>
-      <c r="I16" s="101"/>
+      <c r="I16" s="110"/>
       <c r="J16" s="84"/>
       <c r="K16" s="85" t="s">
         <v>52</v>
@@ -13805,82 +13808,82 @@
       <c r="M16" s="86">
         <v>1</v>
       </c>
-      <c r="N16" s="102">
+      <c r="N16" s="111">
         <v>2</v>
       </c>
-      <c r="O16" s="102"/>
-      <c r="P16" s="102">
+      <c r="O16" s="111"/>
+      <c r="P16" s="111">
         <v>2</v>
       </c>
-      <c r="Q16" s="102"/>
+      <c r="Q16" s="111"/>
       <c r="R16" s="86" t="s">
         <v>76</v>
       </c>
-      <c r="S16" s="102" t="s">
+      <c r="S16" s="111" t="s">
         <v>77</v>
       </c>
-      <c r="T16" s="102"/>
-      <c r="U16" s="102">
+      <c r="T16" s="111"/>
+      <c r="U16" s="111">
         <v>2</v>
       </c>
-      <c r="V16" s="102"/>
+      <c r="V16" s="111"/>
     </row>
     <row r="17" spans="1:22">
-      <c r="A17" s="110" t="s">
+      <c r="A17" s="100" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="103" t="s">
+      <c r="B17" s="96" t="s">
         <v>54</v>
       </c>
-      <c r="C17" s="103" t="s">
+      <c r="C17" s="96" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="103" t="s">
+      <c r="D17" s="96" t="s">
         <v>56</v>
       </c>
-      <c r="E17" s="103"/>
-      <c r="F17" s="103" t="s">
+      <c r="E17" s="96"/>
+      <c r="F17" s="96" t="s">
         <v>78</v>
       </c>
-      <c r="G17" s="103"/>
-      <c r="H17" s="104" t="s">
+      <c r="G17" s="96"/>
+      <c r="H17" s="97" t="s">
         <v>79</v>
       </c>
-      <c r="I17" s="104"/>
+      <c r="I17" s="97"/>
       <c r="J17" s="84"/>
-      <c r="K17" s="107" t="s">
+      <c r="K17" s="104" t="s">
         <v>53</v>
       </c>
-      <c r="L17" s="105" t="s">
+      <c r="L17" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="M17" s="105" t="s">
+      <c r="M17" s="109" t="s">
         <v>55</v>
       </c>
-      <c r="N17" s="105" t="s">
+      <c r="N17" s="109" t="s">
         <v>56</v>
       </c>
-      <c r="O17" s="105"/>
-      <c r="P17" s="105" t="s">
+      <c r="O17" s="109"/>
+      <c r="P17" s="109" t="s">
         <v>78</v>
       </c>
-      <c r="Q17" s="105"/>
-      <c r="R17" s="107" t="s">
+      <c r="Q17" s="109"/>
+      <c r="R17" s="104" t="s">
         <v>52</v>
       </c>
       <c r="S17" s="106" t="s">
         <v>80</v>
       </c>
-      <c r="T17" s="107"/>
-      <c r="U17" s="108" t="s">
+      <c r="T17" s="104"/>
+      <c r="U17" s="105" t="s">
         <v>79</v>
       </c>
-      <c r="V17" s="108"/>
+      <c r="V17" s="105"/>
     </row>
     <row r="18" spans="1:22" ht="24">
-      <c r="A18" s="110"/>
-      <c r="B18" s="103"/>
-      <c r="C18" s="103"/>
+      <c r="A18" s="100"/>
+      <c r="B18" s="96"/>
+      <c r="C18" s="96"/>
       <c r="D18" s="80" t="s">
         <v>81</v>
       </c>
@@ -13900,9 +13903,9 @@
         <v>84</v>
       </c>
       <c r="J18" s="84"/>
-      <c r="K18" s="107"/>
-      <c r="L18" s="105"/>
-      <c r="M18" s="105"/>
+      <c r="K18" s="104"/>
+      <c r="L18" s="109"/>
+      <c r="M18" s="109"/>
       <c r="N18" s="88" t="s">
         <v>81</v>
       </c>
@@ -13915,7 +13918,7 @@
       <c r="Q18" s="88" t="s">
         <v>82</v>
       </c>
-      <c r="R18" s="107"/>
+      <c r="R18" s="104"/>
       <c r="S18" s="88" t="s">
         <v>81</v>
       </c>
@@ -13945,14 +13948,14 @@
       <c r="E19" s="79" t="s">
         <v>88</v>
       </c>
-      <c r="F19" s="109" t="s">
+      <c r="F19" s="112" t="s">
         <v>89</v>
       </c>
-      <c r="G19" s="110"/>
-      <c r="H19" s="110" t="s">
+      <c r="G19" s="100"/>
+      <c r="H19" s="100" t="s">
         <v>90</v>
       </c>
-      <c r="I19" s="110"/>
+      <c r="I19" s="100"/>
       <c r="J19" s="84"/>
       <c r="K19" s="87" t="s">
         <v>85</v>
@@ -13972,7 +13975,7 @@
       <c r="P19" s="106" t="s">
         <v>89</v>
       </c>
-      <c r="Q19" s="107"/>
+      <c r="Q19" s="104"/>
       <c r="R19" s="87" t="s">
         <v>77</v>
       </c>
@@ -13982,10 +13985,10 @@
       <c r="T19" s="87" t="s">
         <v>88</v>
       </c>
-      <c r="U19" s="107" t="s">
+      <c r="U19" s="104" t="s">
         <v>90</v>
       </c>
-      <c r="V19" s="107"/>
+      <c r="V19" s="104"/>
     </row>
     <row r="20" spans="1:22">
       <c r="A20" s="81"/>
@@ -14012,29 +14015,29 @@
       <c r="V20" s="81"/>
     </row>
     <row r="21" spans="1:22">
-      <c r="A21" s="99" t="s">
+      <c r="A21" s="107" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="99"/>
-      <c r="C21" s="99"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="99"/>
-      <c r="F21" s="99"/>
-      <c r="G21" s="99"/>
-      <c r="H21" s="99"/>
+      <c r="B21" s="107"/>
+      <c r="C21" s="107"/>
+      <c r="D21" s="107"/>
+      <c r="E21" s="107"/>
+      <c r="F21" s="107"/>
+      <c r="G21" s="107"/>
+      <c r="H21" s="107"/>
       <c r="I21" s="83"/>
       <c r="J21" s="81"/>
-      <c r="K21" s="100" t="s">
+      <c r="K21" s="108" t="s">
         <v>93</v>
       </c>
-      <c r="L21" s="100"/>
-      <c r="M21" s="100"/>
-      <c r="N21" s="100"/>
-      <c r="O21" s="100"/>
-      <c r="P21" s="100"/>
-      <c r="Q21" s="100"/>
-      <c r="R21" s="100"/>
-      <c r="S21" s="100"/>
+      <c r="L21" s="108"/>
+      <c r="M21" s="108"/>
+      <c r="N21" s="108"/>
+      <c r="O21" s="108"/>
+      <c r="P21" s="108"/>
+      <c r="Q21" s="108"/>
+      <c r="R21" s="108"/>
+      <c r="S21" s="108"/>
       <c r="T21" s="81"/>
       <c r="U21" s="81"/>
       <c r="V21" s="81"/>
@@ -14052,14 +14055,14 @@
       <c r="D22" s="78" t="s">
         <v>76</v>
       </c>
-      <c r="E22" s="101" t="s">
+      <c r="E22" s="110" t="s">
         <v>77</v>
       </c>
-      <c r="F22" s="101"/>
-      <c r="G22" s="101">
+      <c r="F22" s="110"/>
+      <c r="G22" s="110">
         <v>2</v>
       </c>
-      <c r="H22" s="101"/>
+      <c r="H22" s="110"/>
       <c r="I22" s="81"/>
       <c r="J22" s="81"/>
       <c r="K22" s="85" t="s">
@@ -14071,75 +14074,75 @@
       <c r="M22" s="86">
         <v>1</v>
       </c>
-      <c r="N22" s="102">
+      <c r="N22" s="111">
         <v>2</v>
       </c>
-      <c r="O22" s="102"/>
-      <c r="P22" s="102" t="s">
+      <c r="O22" s="111"/>
+      <c r="P22" s="111" t="s">
         <v>94</v>
       </c>
-      <c r="Q22" s="102"/>
-      <c r="R22" s="102">
+      <c r="Q22" s="111"/>
+      <c r="R22" s="111">
         <v>2</v>
       </c>
-      <c r="S22" s="102"/>
+      <c r="S22" s="111"/>
       <c r="T22" s="81"/>
       <c r="U22" s="81"/>
       <c r="V22" s="81"/>
     </row>
     <row r="23" spans="1:22">
-      <c r="A23" s="110" t="s">
+      <c r="A23" s="100" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="104" t="s">
+      <c r="B23" s="97" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="104" t="s">
+      <c r="C23" s="97" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="104" t="s">
+      <c r="D23" s="97" t="s">
         <v>95</v>
       </c>
-      <c r="E23" s="104" t="s">
+      <c r="E23" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="F23" s="104"/>
-      <c r="G23" s="104" t="s">
+      <c r="F23" s="97"/>
+      <c r="G23" s="97" t="s">
         <v>79</v>
       </c>
-      <c r="H23" s="104"/>
+      <c r="H23" s="97"/>
       <c r="I23" s="81"/>
       <c r="J23" s="81"/>
-      <c r="K23" s="107" t="s">
+      <c r="K23" s="104" t="s">
         <v>53</v>
       </c>
-      <c r="L23" s="108" t="s">
+      <c r="L23" s="105" t="s">
         <v>54</v>
       </c>
-      <c r="M23" s="108" t="s">
+      <c r="M23" s="105" t="s">
         <v>55</v>
       </c>
-      <c r="N23" s="108" t="s">
+      <c r="N23" s="105" t="s">
         <v>56</v>
       </c>
-      <c r="O23" s="108"/>
-      <c r="P23" s="105" t="s">
+      <c r="O23" s="105"/>
+      <c r="P23" s="109" t="s">
         <v>78</v>
       </c>
-      <c r="Q23" s="105"/>
-      <c r="R23" s="108" t="s">
+      <c r="Q23" s="109"/>
+      <c r="R23" s="105" t="s">
         <v>79</v>
       </c>
-      <c r="S23" s="108"/>
+      <c r="S23" s="105"/>
       <c r="T23" s="81"/>
       <c r="U23" s="81"/>
       <c r="V23" s="81"/>
     </row>
     <row r="24" spans="1:22" ht="24">
-      <c r="A24" s="110"/>
-      <c r="B24" s="104"/>
-      <c r="C24" s="104"/>
-      <c r="D24" s="104"/>
+      <c r="A24" s="100"/>
+      <c r="B24" s="97"/>
+      <c r="C24" s="97"/>
+      <c r="D24" s="97"/>
       <c r="E24" s="80" t="s">
         <v>81</v>
       </c>
@@ -14154,9 +14157,9 @@
       </c>
       <c r="I24" s="81"/>
       <c r="J24" s="81"/>
-      <c r="K24" s="107"/>
-      <c r="L24" s="108"/>
-      <c r="M24" s="108"/>
+      <c r="K24" s="104"/>
+      <c r="L24" s="105"/>
+      <c r="M24" s="105"/>
       <c r="N24" s="88" t="s">
         <v>81</v>
       </c>
@@ -14192,14 +14195,14 @@
       <c r="D25" s="80" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="104" t="s">
+      <c r="E25" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="F25" s="104"/>
-      <c r="G25" s="104" t="s">
+      <c r="F25" s="97"/>
+      <c r="G25" s="97" t="s">
         <v>90</v>
       </c>
-      <c r="H25" s="104"/>
+      <c r="H25" s="97"/>
       <c r="I25" s="81"/>
       <c r="J25" s="81"/>
       <c r="K25" s="87" t="s">
@@ -14220,11 +14223,11 @@
       <c r="P25" s="106" t="s">
         <v>89</v>
       </c>
-      <c r="Q25" s="107"/>
-      <c r="R25" s="108" t="s">
+      <c r="Q25" s="104"/>
+      <c r="R25" s="105" t="s">
         <v>90</v>
       </c>
-      <c r="S25" s="108"/>
+      <c r="S25" s="105"/>
       <c r="T25" s="81"/>
       <c r="U25" s="81"/>
       <c r="V25" s="81"/>
@@ -14254,26 +14257,26 @@
       <c r="V26" s="81"/>
     </row>
     <row r="27" spans="1:22">
-      <c r="A27" s="99" t="s">
+      <c r="A27" s="107" t="s">
         <v>96</v>
       </c>
-      <c r="B27" s="99"/>
-      <c r="C27" s="99"/>
-      <c r="D27" s="99"/>
-      <c r="E27" s="99"/>
-      <c r="F27" s="99"/>
+      <c r="B27" s="107"/>
+      <c r="C27" s="107"/>
+      <c r="D27" s="107"/>
+      <c r="E27" s="107"/>
+      <c r="F27" s="107"/>
       <c r="G27" s="81"/>
       <c r="H27" s="81"/>
       <c r="I27" s="81"/>
       <c r="J27" s="81"/>
-      <c r="K27" s="100" t="s">
+      <c r="K27" s="108" t="s">
         <v>96</v>
       </c>
-      <c r="L27" s="100"/>
-      <c r="M27" s="100"/>
-      <c r="N27" s="100"/>
-      <c r="O27" s="100"/>
-      <c r="P27" s="100"/>
+      <c r="L27" s="108"/>
+      <c r="M27" s="108"/>
+      <c r="N27" s="108"/>
+      <c r="O27" s="108"/>
+      <c r="P27" s="108"/>
       <c r="Q27" s="81"/>
       <c r="R27" s="81"/>
       <c r="S27" s="81"/>
@@ -14294,10 +14297,10 @@
       <c r="D28" s="77" t="s">
         <v>76</v>
       </c>
-      <c r="E28" s="111" t="s">
+      <c r="E28" s="101" t="s">
         <v>94</v>
       </c>
-      <c r="F28" s="111"/>
+      <c r="F28" s="101"/>
       <c r="G28" s="81"/>
       <c r="H28" s="81"/>
       <c r="I28" s="81"/>
@@ -14314,10 +14317,10 @@
       <c r="N28" s="85" t="s">
         <v>76</v>
       </c>
-      <c r="O28" s="112" t="s">
+      <c r="O28" s="102" t="s">
         <v>94</v>
       </c>
-      <c r="P28" s="112"/>
+      <c r="P28" s="102"/>
       <c r="Q28" s="81"/>
       <c r="R28" s="81"/>
       <c r="S28" s="81"/>
@@ -14326,42 +14329,42 @@
       <c r="V28" s="81"/>
     </row>
     <row r="29" spans="1:22">
-      <c r="A29" s="110" t="s">
+      <c r="A29" s="100" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="104" t="s">
+      <c r="B29" s="97" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="113" t="s">
+      <c r="C29" s="98" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="113" t="s">
+      <c r="D29" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="E29" s="113" t="s">
+      <c r="E29" s="98" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="113"/>
+      <c r="F29" s="98"/>
       <c r="G29" s="81"/>
       <c r="H29" s="81"/>
       <c r="I29" s="81"/>
       <c r="J29" s="81"/>
-      <c r="K29" s="107" t="s">
+      <c r="K29" s="104" t="s">
         <v>53</v>
       </c>
-      <c r="L29" s="108" t="s">
+      <c r="L29" s="105" t="s">
         <v>54</v>
       </c>
-      <c r="M29" s="114" t="s">
+      <c r="M29" s="103" t="s">
         <v>55</v>
       </c>
-      <c r="N29" s="114" t="s">
+      <c r="N29" s="103" t="s">
         <v>68</v>
       </c>
-      <c r="O29" s="114" t="s">
+      <c r="O29" s="103" t="s">
         <v>79</v>
       </c>
-      <c r="P29" s="114"/>
+      <c r="P29" s="103"/>
       <c r="Q29" s="81"/>
       <c r="R29" s="81"/>
       <c r="S29" s="81"/>
@@ -14370,10 +14373,10 @@
       <c r="V29" s="81"/>
     </row>
     <row r="30" spans="1:22" ht="24">
-      <c r="A30" s="110"/>
-      <c r="B30" s="104"/>
-      <c r="C30" s="113"/>
-      <c r="D30" s="113"/>
+      <c r="A30" s="100"/>
+      <c r="B30" s="97"/>
+      <c r="C30" s="98"/>
+      <c r="D30" s="98"/>
       <c r="E30" s="82" t="s">
         <v>83</v>
       </c>
@@ -14384,10 +14387,10 @@
       <c r="H30" s="81"/>
       <c r="I30" s="81"/>
       <c r="J30" s="81"/>
-      <c r="K30" s="107"/>
-      <c r="L30" s="108"/>
-      <c r="M30" s="114"/>
-      <c r="N30" s="114"/>
+      <c r="K30" s="104"/>
+      <c r="L30" s="105"/>
+      <c r="M30" s="103"/>
+      <c r="N30" s="103"/>
       <c r="O30" s="89" t="s">
         <v>83</v>
       </c>
@@ -14432,10 +14435,10 @@
       <c r="N31" s="87" t="s">
         <v>88</v>
       </c>
-      <c r="O31" s="107" t="s">
+      <c r="O31" s="104" t="s">
         <v>90</v>
       </c>
-      <c r="P31" s="107"/>
+      <c r="P31" s="104"/>
       <c r="Q31" s="81"/>
       <c r="R31" s="81"/>
       <c r="S31" s="81"/>
@@ -14459,53 +14462,21 @@
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="K29:K30"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="P25:Q25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="K27:P27"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="M23:M24"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="K21:S21"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="K15:V15"/>
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
     <mergeCell ref="D17:E17"/>
@@ -14522,21 +14493,53 @@
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="H16:I16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="K15:V15"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="P19:Q19"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="K21:S21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="M23:M24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="P25:Q25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="K27:P27"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="D29:D30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19113,7 +19116,7 @@
     <col min="3" max="3" width="5.5703125" style="3" customWidth="1"/>
     <col min="4" max="4" width="7.5703125" style="3" customWidth="1"/>
     <col min="5" max="5" width="5.5703125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="21.5703125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="46.7109375" style="4" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" style="4" customWidth="1"/>
     <col min="8" max="8" width="6.5703125" style="4" customWidth="1"/>
     <col min="9" max="9" width="35.85546875" style="3" customWidth="1"/>
@@ -19484,7 +19487,7 @@
         <v>232</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>792</v>
+        <v>898</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="1" customFormat="1" ht="45">
@@ -19503,7 +19506,7 @@
         <v>112</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>114</v>
@@ -19512,7 +19515,7 @@
         <v>232</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="1" customFormat="1" ht="45">
@@ -19531,7 +19534,7 @@
         <v>112</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>114</v>
@@ -19540,7 +19543,7 @@
         <v>232</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="1" customFormat="1" ht="45">
@@ -19559,7 +19562,7 @@
         <v>112</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>114</v>
@@ -19568,7 +19571,7 @@
         <v>232</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="17" spans="1:20" s="1" customFormat="1">
@@ -19587,16 +19590,16 @@
         <v>112</v>
       </c>
       <c r="F17" s="7" t="s">
+        <v>798</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H17" s="6" t="s">
         <v>799</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H17" s="6" t="s">
+      <c r="I17" s="13" t="s">
         <v>800</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -19615,16 +19618,16 @@
         <v>112</v>
       </c>
       <c r="F18" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="I18" s="13" t="s">
         <v>802</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>800</v>
-      </c>
-      <c r="I18" s="13" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="19" spans="1:20" ht="75">
@@ -19652,7 +19655,7 @@
         <v>88</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -19671,7 +19674,7 @@
         <v>112</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>114</v>
@@ -19680,7 +19683,7 @@
         <v>88</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
@@ -19703,7 +19706,7 @@
         <v>112</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>114</v>
@@ -19712,7 +19715,7 @@
         <v>88</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
@@ -19735,7 +19738,7 @@
         <v>112</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>114</v>
@@ -19744,7 +19747,7 @@
         <v>232</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
@@ -19773,10 +19776,10 @@
         <v>114</v>
       </c>
       <c r="H23" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="I23" s="10" t="s">
         <v>811</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>812</v>
       </c>
       <c r="P23" s="3"/>
       <c r="Q23" s="3"/>
@@ -19799,16 +19802,16 @@
         <v>112</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H24" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="I24" s="10" t="s">
         <v>811</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>812</v>
       </c>
       <c r="P24" s="3"/>
       <c r="Q24" s="3"/>
@@ -19831,7 +19834,7 @@
         <v>112</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>114</v>
@@ -19840,7 +19843,7 @@
         <v>605</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
@@ -19863,7 +19866,7 @@
         <v>112</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>114</v>
@@ -19872,7 +19875,7 @@
         <v>88</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
@@ -19895,7 +19898,7 @@
         <v>112</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="G27" s="10" t="s">
         <v>114</v>
@@ -19904,7 +19907,7 @@
         <v>232</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="28" spans="1:20" s="2" customFormat="1" ht="45">
@@ -19923,16 +19926,16 @@
         <v>112</v>
       </c>
       <c r="F28" s="7" t="s">
+        <v>818</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>810</v>
+      </c>
+      <c r="I28" s="15" t="s">
         <v>819</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>811</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="29" spans="1:20">
@@ -19951,7 +19954,7 @@
         <v>112</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>114</v>
@@ -19960,7 +19963,7 @@
         <v>88</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
@@ -19983,16 +19986,16 @@
         <v>112</v>
       </c>
       <c r="F30" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H30" s="7" t="s">
         <v>822</v>
       </c>
-      <c r="G30" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H30" s="7" t="s">
+      <c r="I30" s="16" t="s">
         <v>823</v>
-      </c>
-      <c r="I30" s="16" t="s">
-        <v>824</v>
       </c>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
@@ -20015,16 +20018,16 @@
         <v>112</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H31" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="I31" s="16" t="s">
         <v>823</v>
-      </c>
-      <c r="I31" s="16" t="s">
-        <v>824</v>
       </c>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
@@ -20047,7 +20050,7 @@
         <v>112</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>114</v>
@@ -20056,7 +20059,7 @@
         <v>88</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
@@ -20079,7 +20082,7 @@
         <v>112</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>114</v>
@@ -20088,7 +20091,7 @@
         <v>88</v>
       </c>
       <c r="I33" s="17" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
@@ -20111,7 +20114,7 @@
         <v>112</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>114</v>
@@ -20120,7 +20123,7 @@
         <v>88</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
@@ -20143,7 +20146,7 @@
         <v>112</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>114</v>
@@ -20152,7 +20155,7 @@
         <v>0.01</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
@@ -20175,7 +20178,7 @@
         <v>112</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>114</v>
@@ -20184,7 +20187,7 @@
         <v>0.01</v>
       </c>
       <c r="I36" s="13" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
@@ -20207,7 +20210,7 @@
         <v>112</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>114</v>
@@ -20216,7 +20219,7 @@
         <v>0.01</v>
       </c>
       <c r="I37" s="13" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
@@ -20239,7 +20242,7 @@
         <v>112</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>114</v>
@@ -20248,7 +20251,7 @@
         <v>88</v>
       </c>
       <c r="I38" s="14" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="P38" s="3"/>
       <c r="Q38" s="3"/>
@@ -20271,7 +20274,7 @@
         <v>112</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>114</v>
@@ -20280,7 +20283,7 @@
         <v>88</v>
       </c>
       <c r="I39" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P39" s="3"/>
       <c r="Q39" s="3"/>
@@ -20303,7 +20306,7 @@
         <v>112</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>114</v>
@@ -20312,7 +20315,7 @@
         <v>88</v>
       </c>
       <c r="I40" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
@@ -20367,7 +20370,7 @@
         <v>112</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>114</v>
@@ -20376,7 +20379,7 @@
         <v>88</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
@@ -20399,7 +20402,7 @@
         <v>112</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>114</v>
@@ -20408,7 +20411,7 @@
         <v>88</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P43" s="3"/>
       <c r="Q43" s="3"/>
@@ -20431,7 +20434,7 @@
         <v>112</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>114</v>
@@ -20440,7 +20443,7 @@
         <v>88</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P44" s="3"/>
       <c r="Q44" s="3"/>
@@ -20463,7 +20466,7 @@
         <v>112</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>114</v>
@@ -20472,7 +20475,7 @@
         <v>88</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P45" s="3"/>
       <c r="Q45" s="3"/>
@@ -20495,7 +20498,7 @@
         <v>112</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>114</v>
@@ -20504,7 +20507,7 @@
         <v>88</v>
       </c>
       <c r="I46" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P46" s="3"/>
       <c r="Q46" s="3"/>
@@ -20527,7 +20530,7 @@
         <v>112</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>114</v>
@@ -20536,7 +20539,7 @@
         <v>88</v>
       </c>
       <c r="I47" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P47" s="3"/>
       <c r="Q47" s="3"/>
@@ -20559,7 +20562,7 @@
         <v>112</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="G48" s="6" t="s">
         <v>114</v>
@@ -20568,7 +20571,7 @@
         <v>88</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P48" s="3"/>
       <c r="Q48" s="3"/>
@@ -20591,7 +20594,7 @@
         <v>112</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="G49" s="6" t="s">
         <v>114</v>
@@ -20600,7 +20603,7 @@
         <v>88</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="P49" s="3"/>
       <c r="Q49" s="3"/>
@@ -20623,16 +20626,16 @@
         <v>112</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="G50" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H50" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="I50" s="17" t="s">
         <v>823</v>
-      </c>
-      <c r="I50" s="17" t="s">
-        <v>824</v>
       </c>
       <c r="P50" s="3"/>
       <c r="Q50" s="3"/>
@@ -20655,7 +20658,7 @@
         <v>112</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="G51" s="6" t="s">
         <v>114</v>
@@ -20664,7 +20667,7 @@
         <v>88</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="P51" s="3"/>
       <c r="Q51" s="3"/>
@@ -20687,7 +20690,7 @@
         <v>112</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="G52" s="6" t="s">
         <v>114</v>
@@ -20696,7 +20699,7 @@
         <v>88</v>
       </c>
       <c r="I52" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="53" spans="1:20">
@@ -20715,7 +20718,7 @@
         <v>112</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="G53" s="6" t="s">
         <v>114</v>
@@ -20724,7 +20727,7 @@
         <v>88</v>
       </c>
       <c r="I53" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="54" spans="1:20">
@@ -20743,7 +20746,7 @@
         <v>112</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>114</v>
@@ -20752,7 +20755,7 @@
         <v>88</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="55" spans="1:20">
@@ -20771,16 +20774,16 @@
         <v>112</v>
       </c>
       <c r="F55" s="7" t="s">
+        <v>854</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H55" s="7" t="s">
         <v>855</v>
       </c>
-      <c r="G55" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H55" s="7" t="s">
+      <c r="I55" s="16" t="s">
         <v>856</v>
-      </c>
-      <c r="I55" s="16" t="s">
-        <v>857</v>
       </c>
     </row>
     <row r="56" spans="1:20">
@@ -20805,10 +20808,10 @@
         <v>114</v>
       </c>
       <c r="H56" s="7" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="I56" s="16" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="P56" s="3"/>
       <c r="Q56" s="3"/>
@@ -20837,10 +20840,10 @@
         <v>114</v>
       </c>
       <c r="H57" s="7" t="s">
+        <v>857</v>
+      </c>
+      <c r="I57" s="16" t="s">
         <v>858</v>
-      </c>
-      <c r="I57" s="16" t="s">
-        <v>859</v>
       </c>
       <c r="P57" s="3"/>
       <c r="Q57" s="3"/>
@@ -20872,7 +20875,7 @@
         <v>88</v>
       </c>
       <c r="I58" s="16" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="P58" s="3"/>
       <c r="Q58" s="3"/>
@@ -20904,7 +20907,7 @@
         <v>88</v>
       </c>
       <c r="I59" s="16" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="P59" s="3"/>
       <c r="Q59" s="3"/>
@@ -20936,7 +20939,7 @@
         <v>88</v>
       </c>
       <c r="I60" s="16" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="P60" s="3"/>
       <c r="Q60" s="3"/>
@@ -20959,16 +20962,16 @@
         <v>112</v>
       </c>
       <c r="F61" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H61" s="6" t="s">
         <v>863</v>
       </c>
-      <c r="G61" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H61" s="6" t="s">
-        <v>864</v>
-      </c>
       <c r="I61" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P61" s="3"/>
       <c r="Q61" s="3"/>
@@ -20991,16 +20994,16 @@
         <v>112</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="G62" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I62" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
@@ -21023,16 +21026,16 @@
         <v>112</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="G63" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I63" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P63" s="3"/>
       <c r="Q63" s="3"/>
@@ -21055,16 +21058,16 @@
         <v>112</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="G64" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I64" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P64" s="3"/>
       <c r="Q64" s="3"/>
@@ -21087,16 +21090,16 @@
         <v>112</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G65" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I65" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P65" s="3"/>
       <c r="Q65" s="3"/>
@@ -21119,16 +21122,16 @@
         <v>112</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I66" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P66" s="3"/>
       <c r="Q66" s="3"/>
@@ -21150,14 +21153,14 @@
         <v>112</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G67" s="6" t="s">
         <v>114</v>
       </c>
       <c r="H67" s="6"/>
       <c r="I67" s="17" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="P67" s="3"/>
       <c r="Q67" s="3"/>
@@ -21180,14 +21183,14 @@
         <v>112</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G68" s="8" t="s">
         <v>114</v>
       </c>
       <c r="H68" s="17"/>
       <c r="I68" s="17" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="P68" s="3"/>
       <c r="Q68" s="3"/>
@@ -21215,10 +21218,10 @@
         <v>114</v>
       </c>
       <c r="H69" s="4" t="s">
+        <v>873</v>
+      </c>
+      <c r="I69" s="21" t="s">
         <v>874</v>
-      </c>
-      <c r="I69" s="21" t="s">
-        <v>875</v>
       </c>
       <c r="P69" s="3"/>
       <c r="Q69" s="3"/>
@@ -21239,13 +21242,13 @@
         <v>112</v>
       </c>
       <c r="F70" s="4" t="s">
+        <v>875</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="I70" s="21" t="s">
         <v>876</v>
-      </c>
-      <c r="G70" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="I70" s="21" t="s">
-        <v>877</v>
       </c>
       <c r="P70" s="3"/>
       <c r="Q70" s="3"/>
@@ -21266,16 +21269,16 @@
         <v>112</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="G71" s="8" t="s">
         <v>114</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I71" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P71" s="3"/>
       <c r="Q71" s="3"/>
@@ -21296,16 +21299,16 @@
         <v>112</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="G72" s="8" t="s">
         <v>114</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="I72" s="16" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="P72" s="3"/>
       <c r="Q72" s="3"/>
@@ -21326,16 +21329,16 @@
         <v>112</v>
       </c>
       <c r="F73" s="19" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>114</v>
       </c>
       <c r="H73" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="I73" s="16" t="s">
         <v>823</v>
-      </c>
-      <c r="I73" s="16" t="s">
-        <v>824</v>
       </c>
       <c r="P73" s="3"/>
       <c r="Q73" s="3"/>
@@ -21356,16 +21359,16 @@
         <v>112</v>
       </c>
       <c r="F74" s="19" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>114</v>
       </c>
       <c r="H74" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="I74" s="16" t="s">
         <v>823</v>
-      </c>
-      <c r="I74" s="16" t="s">
-        <v>824</v>
       </c>
       <c r="P74" s="3"/>
       <c r="Q74" s="3"/>
@@ -21387,14 +21390,14 @@
         <v>112</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G75" s="2" t="s">
         <v>114</v>
       </c>
       <c r="H75" s="2"/>
       <c r="I75" s="20" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="L75" s="21"/>
       <c r="P75" s="3"/>
@@ -21416,7 +21419,7 @@
         <v>112</v>
       </c>
       <c r="F76" s="18" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>114</v>
@@ -21425,7 +21428,7 @@
         <v>234</v>
       </c>
       <c r="I76" s="21" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="P76" s="3"/>
       <c r="Q76" s="3"/>
@@ -21440,19 +21443,19 @@
         <v>16714</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>112</v>
       </c>
       <c r="F77" s="18" t="s">
+        <v>886</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I77" s="21" t="s">
         <v>887</v>
-      </c>
-      <c r="G77" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I77" s="21" t="s">
-        <v>888</v>
       </c>
       <c r="P77" s="3"/>
       <c r="Q77" s="3"/>
@@ -21467,19 +21470,19 @@
         <v>16715</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>112</v>
       </c>
       <c r="F78" s="18" t="s">
+        <v>889</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I78" s="21" t="s">
         <v>890</v>
-      </c>
-      <c r="G78" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I78" s="21" t="s">
-        <v>891</v>
       </c>
       <c r="P78" s="3"/>
       <c r="Q78" s="3"/>
@@ -21494,19 +21497,19 @@
         <v>16715</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>112</v>
       </c>
       <c r="F79" s="18" t="s">
+        <v>892</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I79" s="21" t="s">
         <v>893</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I79" s="21" t="s">
-        <v>894</v>
       </c>
       <c r="P79" s="3"/>
       <c r="Q79" s="3"/>
@@ -22128,7 +22131,7 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="22" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="B23" s="23">
         <f t="shared" si="0"/>
@@ -22154,7 +22157,7 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="22" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B24" s="23">
         <f t="shared" si="0"/>
@@ -22180,7 +22183,7 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="22" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B25" s="23">
         <f t="shared" si="0"/>
@@ -22206,7 +22209,7 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="22" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="B26" s="23">
         <f t="shared" si="0"/>
@@ -32340,7 +32343,7 @@
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="5.5703125" customWidth="1"/>
     <col min="4" max="4" width="7.5703125" customWidth="1"/>
-    <col min="5" max="5" width="5.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" customWidth="1"/>
     <col min="6" max="6" width="27.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.5703125" style="23" customWidth="1"/>
     <col min="8" max="8" width="5.5703125" customWidth="1"/>

</xml_diff>